<commit_message>
feat: acceptance criteria field + baseline quality evaluation + feature extraction pipeline
Major changes:
- Add acceptance_criteria field across full pipeline (Excel→parse→extract→report)
- Implement baseline quality evaluation with statistical gradient/attribution checks
- Build LLM-based feature extraction pipeline replacing raw text embedding
- Add batch estimate with Excel import/export support
- Add split suggestion for stories exceeding 13 points
- Template upgraded from 4-column to 5-column (ID/标题/描述/验收标准/故事点)
- SQLite migration for existing databases with ALTER TABLE
</commit_message>
<xml_diff>
--- a/story point/static/baseline_template.xlsx
+++ b/story point/static/baseline_template.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,13 +434,18 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>验收标准</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>故事点</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="无效的故事点" error="请选择有效的故事点: 1, 2, 3, 5, 8, 13" type="list">
+    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="无效的故事点" error="请选择有效的故事点: 1, 2, 3, 5, 8, 13" type="list">
       <formula1>"1,2,3,5,8,13"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>